<commit_message>
slurry data for january experiment written
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-data.xlsx
+++ b/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-01-06-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82E09F8-7021-42C3-B4C7-C293B6C8AE5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0600709F-3C4F-4A13-8A24-390AA57E06C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-2820" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,15 +26,173 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Mikael Løvig Larsen</author>
+  </authors>
+  <commentList>
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{83D0CFFF-C029-459E-9523-597C936FA63D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Mikael Løvig Larsen:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+no container mass</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>triplicate measurements on same sample at different locations</t>
+  </si>
+  <si>
+    <t>Treatment</t>
+  </si>
+  <si>
+    <t>AA</t>
+  </si>
+  <si>
+    <t>H2SO4</t>
+  </si>
+  <si>
+    <t>Untreated</t>
+  </si>
+  <si>
+    <t>V acid [mL]</t>
+  </si>
+  <si>
+    <t>pH before</t>
+  </si>
+  <si>
+    <t>500 g slurry acidified for each treatment</t>
+  </si>
+  <si>
+    <t>pH after</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>pH before exp</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>untreated1</t>
+  </si>
+  <si>
+    <t>untreated2</t>
+  </si>
+  <si>
+    <t>untreated3</t>
+  </si>
+  <si>
+    <t>AA1</t>
+  </si>
+  <si>
+    <t>AA2</t>
+  </si>
+  <si>
+    <t>AA3</t>
+  </si>
+  <si>
+    <t>H2SO4 1</t>
+  </si>
+  <si>
+    <t>H2SO4 2</t>
+  </si>
+  <si>
+    <t>H2SO4 3</t>
+  </si>
+  <si>
+    <t>STD 1</t>
+  </si>
+  <si>
+    <t>STD 2</t>
+  </si>
+  <si>
+    <t>m(slurry) [g]</t>
+  </si>
+  <si>
+    <t>49 mL of water for slurry samples</t>
+  </si>
+  <si>
+    <t>24.5 for stds</t>
+  </si>
+  <si>
+    <t>NH4 measurement [mg/L]</t>
+  </si>
+  <si>
+    <t>41*</t>
+  </si>
+  <si>
+    <t>Crucible nr</t>
+  </si>
+  <si>
+    <t>m(sample, wet) [g]</t>
+  </si>
+  <si>
+    <t>m(container) [g]</t>
+  </si>
+  <si>
+    <t>Untr</t>
+  </si>
+  <si>
+    <t>Decription</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="167" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,8 +215,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -339,27 +500,430 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="56.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="E2">
+        <v>7.06</v>
+      </c>
+      <c r="F2">
+        <v>6.22</v>
+      </c>
+      <c r="G2">
+        <v>6.39</v>
+      </c>
+      <c r="H2" s="1">
+        <v>6.4</v>
+      </c>
+      <c r="I2" s="1">
+        <v>6.39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>0.79</v>
+      </c>
+      <c r="E3">
+        <v>7.09</v>
+      </c>
+      <c r="F3">
+        <v>6.23</v>
+      </c>
+      <c r="G3">
+        <v>6.43</v>
+      </c>
+      <c r="H3">
+        <v>6.41</v>
+      </c>
+      <c r="I3">
+        <v>6.41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>6.95</v>
+      </c>
+      <c r="F4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>7.04</v>
+      </c>
+      <c r="H4">
+        <v>7.04</v>
+      </c>
+      <c r="I4">
+        <v>7.04</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F7390D-8C65-402E-B031-C0A94901E7D3}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>1.0589</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>1.0946</v>
+      </c>
+      <c r="E3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>1.0609999999999999</v>
+      </c>
+      <c r="E4">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>1.0511999999999999</v>
+      </c>
+      <c r="E5">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6">
+        <v>1.0470999999999999</v>
+      </c>
+      <c r="E6">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7">
+        <v>1.0250999999999999</v>
+      </c>
+      <c r="E7">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8">
+        <v>1.0347999999999999</v>
+      </c>
+      <c r="E8">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1.0647</v>
+      </c>
+      <c r="E9">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10">
+        <v>1.0263</v>
+      </c>
+      <c r="E10">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0.49199999999999999</v>
+      </c>
+      <c r="E11">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12">
+        <v>0.49830000000000002</v>
+      </c>
+      <c r="E12">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2D6C95A-479E-4C84-94F4-777190CE73FB}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2D6C95A-479E-4C84-94F4-777190CE73FB}">
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C2">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="3">
+        <v>30.201000000000001</v>
+      </c>
+      <c r="F2">
+        <v>31.996500000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C3">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3">
+        <v>31.4588</v>
+      </c>
+      <c r="F3">
+        <v>34.002499999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4">
+        <v>31.767600000000002</v>
+      </c>
+      <c r="F4">
+        <v>33.357100000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>32.648000000000003</v>
+      </c>
+      <c r="F5">
+        <v>34.054900000000004</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>30.0655</v>
+      </c>
+      <c r="F6">
+        <v>33.6218</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C7">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>30.7576</v>
+      </c>
+      <c r="F7">
+        <v>35.097200000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C8">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>34.088799999999999</v>
+      </c>
+      <c r="F8">
+        <v>33.154800000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <v>212</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="2">
+        <v>37.302900000000001</v>
+      </c>
+      <c r="F9">
+        <v>31.262699999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C10">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>37.472499999999997</v>
+      </c>
+      <c r="F10">
+        <v>34.545499999999997</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lab pig slurry tests data
Added test-data from the lab pig slurry exp

also edited comments in interpolation-integration v2
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-data.xlsx
+++ b/Lab-trails/2026-01-06-cattle-slurry/2026-01-06-cattle-slurry-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-01-06-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091B6FE7-6EEE-4B5D-9F5A-A43EB8007429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0E3AB6-B288-4E28-96C5-68B8175BEA6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pH" sheetId="1" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
   <si>
     <t>Description</t>
   </si>
@@ -216,6 +216,9 @@
   </si>
   <si>
     <t>m(crucible) [g]</t>
+  </si>
+  <si>
+    <t>expected weight</t>
   </si>
 </sst>
 </file>
@@ -699,18 +702,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F7390D-8C65-402E-B031-C0A94901E7D3}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -721,16 +724,19 @@
         <v>24</v>
       </c>
       <c r="E1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" t="s">
         <v>27</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>32</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -741,17 +747,20 @@
         <v>1.0589</v>
       </c>
       <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>41</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>50</v>
       </c>
-      <c r="G2" s="1">
-        <f>((E2*F2)/D2)/1000</f>
+      <c r="H2" s="1">
+        <f>((F2*G2*E2)/D2)/1000</f>
         <v>1.9359712909623195</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -762,17 +771,20 @@
         <v>1.0946</v>
       </c>
       <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>44</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>50</v>
       </c>
-      <c r="G3" s="1">
-        <f t="shared" ref="G3:G12" si="0">((E3*F3)/D3)/1000</f>
+      <c r="H3" s="1">
+        <f t="shared" ref="H3:H12" si="0">((F3*G3*E3)/D3)/1000</f>
         <v>2.0098666179426274</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>15</v>
       </c>
@@ -780,17 +792,20 @@
         <v>1.0609999999999999</v>
       </c>
       <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>41</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>50</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <f t="shared" si="0"/>
         <v>1.9321394910461829</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>16</v>
       </c>
@@ -798,17 +813,20 @@
         <v>1.0511999999999999</v>
       </c>
       <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>39</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>50</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <f t="shared" si="0"/>
         <v>1.8550228310502284</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>17</v>
       </c>
@@ -816,17 +834,20 @@
         <v>1.0470999999999999</v>
       </c>
       <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>38</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>50</v>
       </c>
-      <c r="G6" s="1">
+      <c r="H6" s="1">
         <f t="shared" si="0"/>
         <v>1.8145353834399773</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>18</v>
       </c>
@@ -834,17 +855,20 @@
         <v>1.0250999999999999</v>
       </c>
       <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
         <v>39</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>50</v>
       </c>
-      <c r="G7" s="1">
+      <c r="H7" s="1">
         <f t="shared" si="0"/>
         <v>1.9022534386889085</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>19</v>
       </c>
@@ -852,17 +876,20 @@
         <v>1.0347999999999999</v>
       </c>
       <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
         <v>39</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>50</v>
       </c>
-      <c r="G8" s="1">
+      <c r="H8" s="1">
         <f t="shared" si="0"/>
         <v>1.8844221105527641</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>20</v>
       </c>
@@ -870,17 +897,20 @@
         <v>1.0647</v>
       </c>
       <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
         <v>36</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>50</v>
       </c>
-      <c r="G9" s="1">
+      <c r="H9" s="1">
         <f t="shared" si="0"/>
         <v>1.6906170752324599</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
         <v>21</v>
       </c>
@@ -888,17 +918,20 @@
         <v>1.0263</v>
       </c>
       <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>39</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>50</v>
       </c>
-      <c r="G10" s="1">
+      <c r="H10" s="1">
         <f t="shared" si="0"/>
         <v>1.900029231218942</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>22</v>
       </c>
@@ -906,17 +939,20 @@
         <v>0.49199999999999999</v>
       </c>
       <c r="E11">
+        <v>0.5</v>
+      </c>
+      <c r="F11">
         <v>67</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>50</v>
       </c>
-      <c r="G11" s="1">
-        <f t="shared" si="0"/>
-        <v>6.808943089430894</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11" s="1">
+        <f t="shared" si="0"/>
+        <v>3.404471544715447</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
         <v>23</v>
       </c>
@@ -924,14 +960,17 @@
         <v>0.49830000000000002</v>
       </c>
       <c r="E12">
+        <v>0.5</v>
+      </c>
+      <c r="F12">
         <v>57</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>50</v>
       </c>
-      <c r="G12" s="1">
-        <f t="shared" si="0"/>
-        <v>5.7194461167971102</v>
+      <c r="H12" s="1">
+        <f t="shared" si="0"/>
+        <v>2.8597230583985551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>